<commit_message>
Improve adaptive learning and assessment workflows
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/SmartPlay_Simple_Assessment_Template.xlsx
+++ b/backend/src/main/resources/templates/SmartPlay_Simple_Assessment_Template.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assessment Scores'!$A$1:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assessment Scores'!$A$1:$L$501</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Student Name</t>
   </si>
@@ -66,7 +66,7 @@
     <t>Kavindu Perera</t>
   </si>
   <si>
-    <t>School ID</t>
+    <t>Student ID</t>
   </si>
   <si>
     <t>Ayesha Niyas</t>
@@ -115,6 +115,15 @@
   </si>
   <si>
     <t>Thehan Rodrigo</t>
+  </si>
+  <si>
+    <t>Attempts</t>
+  </si>
+  <si>
+    <t>Time Taken (Minutes)</t>
+  </si>
+  <si>
+    <t>Completion Status</t>
   </si>
 </sst>
 </file>
@@ -472,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -483,6 +492,9 @@
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="9" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -512,6 +524,15 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>